<commit_message>
Rebuild No-L order on 14d basis (Variant A): corrections for non-incoming items, blogger MOQ noted
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FAj7riRQuseKrZcipVDuEw
</commit_message>
<xml_diff>
--- a/Таблицы/Заказ_NoL_2026-06-30.xlsx
+++ b/Таблицы/Заказ_NoL_2026-06-30.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Заказ No-L" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Заказ No-L (14д)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
@@ -68,14 +72,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,174 +446,133 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Заказ No-L из Китая · база Расчётный 14д · выкупы 🟢/🟡 · бюджет 50 000 ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Выкупы</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Бренд</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Название</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Размер</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Штрихкод</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Артикул WB</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Артикул Ozon</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Заказы 28д</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Нужно (расч.28д)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Общий остаток</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Нужно (14д)</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>К заказу, шт</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Себест. ₽/шт</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Сумма ₽</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>зелёный</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>MSH</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Сережки «Мишель»</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Серьги</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2038819575882</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>MSH-021</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>MSH-021</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>18</v>
-      </c>
-      <c r="K2" t="n">
-        <v>5</v>
-      </c>
-      <c r="L2" t="n">
-        <v>5</v>
-      </c>
-      <c r="M2" t="n">
-        <v>245</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1225</v>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DSS</t>
+          <t>MSH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Сережки «Перламутровое сердце»</t>
+          <t>Сережки «Мишель»</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -623,100 +587,112 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2037549815565</t>
+          <t>2038819575882</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>D275DSR107</t>
+          <t>MSH-021</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>D238</t>
+          <t>MSH-021</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K3" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
         <v>18</v>
       </c>
       <c r="M3" t="n">
-        <v>350</v>
+        <v>18</v>
       </c>
       <c r="N3" t="n">
-        <v>6300</v>
-      </c>
+        <v>245</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4410</v>
+      </c>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MSH</t>
+          <t>DSS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Колье «Солнце»</t>
+          <t>Сережки «Перламутровое сердце»</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Колье</t>
+          <t>Серьги</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>44-49</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2038819637474</t>
+          <t>2037549815565</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>MSHK-032</t>
+          <t>D275DSR107</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>MSHK-032</t>
+          <t>D238</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="M4" t="n">
-        <v>159</v>
+        <v>28</v>
       </c>
       <c r="N4" t="n">
-        <v>477</v>
+        <v>350</v>
+      </c>
+      <c r="O4" t="n">
+        <v>9800</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>пересчёт: приход не в пути</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
@@ -728,55 +704,59 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Сережки «Ласточкины сны»</t>
+          <t>Колье «Счастливая звезда»</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Серьги</t>
+          <t>Колье</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>40-45</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2043835932274</t>
+          <t>2038819637481</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>MSH-089</t>
+          <t>MSHK-033</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>MSH-089</t>
+          <t>MSHK-033</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="L5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M5" t="n">
-        <v>315</v>
+        <v>3</v>
       </c>
       <c r="N5" t="n">
-        <v>2520</v>
-      </c>
+        <v>162</v>
+      </c>
+      <c r="O5" t="n">
+        <v>486</v>
+      </c>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
@@ -788,55 +768,59 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Сережки «Джулианна»</t>
+          <t>Колье «Солнце»</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Серьги</t>
+          <t>Колье</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>44-49</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2039500932724</t>
+          <t>2038819637474</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>MSHK-047</t>
+          <t>MSHK-032</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>MSHK-047</t>
+          <t>MSHK-032</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M6" t="n">
-        <v>132</v>
+        <v>6</v>
       </c>
       <c r="N6" t="n">
-        <v>660</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="O6" t="n">
+        <v>954</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
@@ -848,55 +832,59 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Колье «Алма»</t>
+          <t>Сережки «Ласточкины сны»</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Колье</t>
+          <t>Серьги</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>42-47</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2038819637351</t>
+          <t>2043835932274</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>MSHK-028</t>
+          <t>MSH-089</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>MSHK-028</t>
+          <t>MSH-089</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K7" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="L7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M7" t="n">
-        <v>483</v>
+        <v>15</v>
       </c>
       <c r="N7" t="n">
-        <v>7728</v>
-      </c>
+        <v>315</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4725</v>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
@@ -908,7 +896,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Сережки «Ариэлла»</t>
+          <t>Сережки «Джулианна»</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -923,100 +911,108 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2039500932694</t>
+          <t>2039500932724</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>MSHK-040</t>
+          <t>MSHK-047</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>MSHK-040</t>
+          <t>MSHK-047</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="L8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M8" t="n">
-        <v>145</v>
+        <v>9</v>
       </c>
       <c r="N8" t="n">
-        <v>145</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1188</v>
+      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>зелёный</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MSH</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Колье «Алма»</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Колье</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>42-47</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2038819637351</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>MSHK-028</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>MSHK-028</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>зелёный</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>MSH</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Колье «Счастливое число 7»</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Колье</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>40-45</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2038819637429</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>MSHK-029</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>MSHK-029</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>6</v>
       </c>
-      <c r="K9" t="n">
-        <v>5</v>
-      </c>
       <c r="L9" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="M9" t="n">
-        <v>128</v>
+        <v>19</v>
       </c>
       <c r="N9" t="n">
-        <v>640</v>
-      </c>
+        <v>483</v>
+      </c>
+      <c r="O9" t="n">
+        <v>9177</v>
+      </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
@@ -1028,7 +1024,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Сережки «Рената»</t>
+          <t>Сережки «Ариэлла»</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1043,242 +1039,655 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2042109116037</t>
+          <t>2039500932694</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>MSH-069</t>
+          <t>MSHK-040</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>MSH-069</t>
+          <t>MSHK-040</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K10" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="L10" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="M10" t="n">
-        <v>412</v>
+        <v>2</v>
       </c>
       <c r="N10" t="n">
-        <v>5356</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="O10" t="n">
+        <v>290</v>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>зелёный</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DSS</t>
+          <t>MSH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Колье «Фрэнсис»</t>
+          <t>Сережки «Рената»</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Колье</t>
+          <t>Серьги</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>40-45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2042109298498</t>
+          <t>2042109116037</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>D506</t>
+          <t>MSH-069</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>D506</t>
+          <t>MSH-069</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M11" t="n">
-        <v>620</v>
+        <v>7</v>
       </c>
       <c r="N11" t="n">
-        <v>3720</v>
-      </c>
+        <v>412</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2884</v>
+      </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>зелёный</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DSS</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Колье «Фрэнсис»</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Колье</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>40-45</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2042109298498</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>D506</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>D506</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>зелёный</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>MSH</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Сережки «Барбара»</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Серьги</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2042109156897</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>MSH-072</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>MSH-072</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>3</v>
-      </c>
-      <c r="K12" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" t="n">
-        <v>3</v>
-      </c>
       <c r="M12" t="n">
-        <v>173</v>
+        <v>11</v>
       </c>
       <c r="N12" t="n">
-        <v>519</v>
-      </c>
+        <v>620</v>
+      </c>
+      <c r="O12" t="n">
+        <v>6820</v>
+      </c>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>зелёный</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MSH</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Сережки «Барбара»</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Серьги</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2042109156897</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>MSH-072</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>MSH-072</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" t="n">
+        <v>14</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" t="n">
+        <v>173</v>
+      </c>
+      <c r="O13" t="n">
+        <v>346</v>
+      </c>
+      <c r="P13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>зелёный</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DSS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Сережки «Иветта»</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Серьги</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2043834127534</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>D515</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>D515</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" t="n">
+        <v>8</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>795</v>
+      </c>
+      <c r="O14" t="n">
+        <v>795</v>
+      </c>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>жёлтый</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>MSH</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Колье с двумя кулонами «Римские истории»</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Сережки «Амели»</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Серьги</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2038819575851</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>MSH-018</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>MSH-018</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>17</v>
+      </c>
+      <c r="K15" t="n">
+        <v>16</v>
+      </c>
+      <c r="L15" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" t="n">
+        <v>213</v>
+      </c>
+      <c r="O15" t="n">
+        <v>852</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>пересчёт: приход не в пути</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>жёлтый</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MSH</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Сережки «Сирень»</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Серьги</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2038819575769</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>MSH-009</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>MSH-009</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>13</v>
+      </c>
+      <c r="K16" t="n">
+        <v>27</v>
+      </c>
+      <c r="L16" t="n">
+        <v>7</v>
+      </c>
+      <c r="M16" t="n">
+        <v>7</v>
+      </c>
+      <c r="N16" t="n">
+        <v>178</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1246</v>
+      </c>
+      <c r="P16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>жёлтый</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MSH</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Сережки «Цветочные истории»</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Серьги</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2038819575684</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>MSH-001</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>MSH-001</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>12</v>
+      </c>
+      <c r="K17" t="n">
+        <v>29</v>
+      </c>
+      <c r="L17" t="n">
+        <v>6</v>
+      </c>
+      <c r="M17" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" t="n">
+        <v>412</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2472</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>жёлтый</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DSS</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Сережки «Клевер»</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Серьги</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2031764978623</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>D175DSR035</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>D176</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>9</v>
+      </c>
+      <c r="K18" t="n">
+        <v>11</v>
+      </c>
+      <c r="L18" t="n">
+        <v>19</v>
+      </c>
+      <c r="M18" t="n">
+        <v>19</v>
+      </c>
+      <c r="N18" t="n">
+        <v>170</v>
+      </c>
+      <c r="O18" t="n">
+        <v>3230</v>
+      </c>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>жёлтый</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DSS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Колье «Триша»</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Колье</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>37-42</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2038819637283</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>MSHK-027</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>MSHK-027</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>85</v>
-      </c>
-      <c r="K13" t="n">
-        <v>142</v>
-      </c>
-      <c r="L13" t="n">
-        <v>104</v>
-      </c>
-      <c r="M13" t="n">
-        <v>199</v>
-      </c>
-      <c r="N13" t="n">
-        <v>20696</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2037853259284</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>D184DKLE012</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>D310</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>7</v>
+      </c>
+      <c r="K19" t="n">
+        <v>14</v>
+      </c>
+      <c r="L19" t="n">
+        <v>6</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>175</v>
+      </c>
+      <c r="O19" t="n">
+        <v>175</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>частично по бюджету</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="4" t="n">
-        <v>225</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>187</v>
-      </c>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="n">
-        <v>49986</v>
-      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="n">
+        <v>163</v>
+      </c>
+      <c r="M20" s="5" t="n">
+        <v>158</v>
+      </c>
+      <c r="N20" s="5" t="inlineStr"/>
+      <c r="O20" s="5" t="n">
+        <v>49850</v>
+      </c>
+      <c r="P20" s="5" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Ромашки (10) and Римские истории (100) to order; budget extended to 71950
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FAj7riRQuseKrZcipVDuEw
</commit_message>
<xml_diff>
--- a/Таблицы/Заказ_NoL_2026-06-30.xlsx
+++ b/Таблицы/Заказ_NoL_2026-06-30.xlsx
@@ -37,7 +37,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -72,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -80,6 +85,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -446,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -464,13 +470,13 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Заказ No-L из Китая · база Расчётный 14д · выкупы 🟢/🟡 · бюджет 50 000 ₽</t>
+          <t>Заказ No-L из Китая · база Расчётный 14д · Вариант A + ручные добавления · 71950 ₽</t>
         </is>
       </c>
     </row>
@@ -1652,41 +1658,175 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>частично по бюджету</t>
+          <t>частично (нужно 6)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>жёлтый</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MSH</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Колье с двумя кулонами «Римские истории»</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Колье</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>37-42</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2038819637283</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>MSHK-027</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>MSHK-027</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>85</v>
+      </c>
+      <c r="K20" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" t="n">
+        <v>94</v>
+      </c>
+      <c r="M20" t="n">
+        <v>100</v>
+      </c>
+      <c r="N20" t="n">
+        <v>199</v>
+      </c>
+      <c r="O20" t="n">
+        <v>19900</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>добавлено вручную (MOQ 100; спрос блогерский)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>красный</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MSH</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Сережки «Ромашки»</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Серьги</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2039500932779</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>MSHK-052</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>MSHK-052</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>16</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>10</v>
+      </c>
+      <c r="N21" t="n">
+        <v>220</v>
+      </c>
+      <c r="O21" t="n">
+        <v>2200</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>добавлено вручную (выкуп 🔴; запаса ~56 дн)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr"/>
+      <c r="B22" s="6" t="inlineStr"/>
+      <c r="C22" s="6" t="inlineStr"/>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="5" t="n">
-        <v>163</v>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>158</v>
-      </c>
-      <c r="N20" s="5" t="inlineStr"/>
-      <c r="O20" s="5" t="n">
-        <v>49850</v>
-      </c>
-      <c r="P20" s="5" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
+      <c r="M22" s="6" t="n">
+        <v>268</v>
+      </c>
+      <c r="N22" s="6" t="inlineStr"/>
+      <c r="O22" s="6" t="n">
+        <v>71950</v>
+      </c>
+      <c r="P22" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>